<commit_message>
Added aging + FCRN
</commit_message>
<xml_diff>
--- a/Data/Charging_point_test_data.xlsx
+++ b/Data/Charging_point_test_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\araavind\Desktop\Python Files\LEC-Opt\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/araavind/Desktop/Python Files/LEC-Opt/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D06D1A8C-C164-4F12-ACB5-5B653F332FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41683461-30D7-6D45-9870-57610E323F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D862B17B-82BE-45C1-B5E7-E58196152A87}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17180" activeTab="1" xr2:uid="{D862B17B-82BE-45C1-B5E7-E58196152A87}"/>
   </bookViews>
   <sheets>
     <sheet name="CP1" sheetId="1" r:id="rId1"/>
@@ -431,15 +431,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D0C6441-60F9-4825-A4B9-DE936FF6AEE4}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -462,7 +462,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>50</v>
       </c>
@@ -476,7 +476,7 @@
         <v>44927.208333333336</v>
       </c>
       <c r="E2">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -485,7 +485,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>65</v>
       </c>
@@ -499,7 +499,7 @@
         <v>44927.625</v>
       </c>
       <c r="E3">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -508,7 +508,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>70</v>
       </c>
@@ -522,7 +522,7 @@
         <v>44927.958333333336</v>
       </c>
       <c r="E4">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="F4">
         <v>0.8</v>
@@ -539,15 +539,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{144132FB-CE19-480F-9174-B11643F453D0}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -570,7 +570,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>50</v>
       </c>
@@ -587,13 +587,13 @@
         <v>0.7</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G2">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>65</v>
       </c>
@@ -610,13 +610,13 @@
         <v>0.5</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="G3">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>70</v>
       </c>
@@ -633,13 +633,13 @@
         <v>0.6</v>
       </c>
       <c r="F4">
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="G4">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>50</v>
       </c>
@@ -656,13 +656,13 @@
         <v>0.7</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="G5">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>65</v>
       </c>
@@ -679,13 +679,13 @@
         <v>0.5</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="G6">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>70</v>
       </c>

</xml_diff>

<commit_message>
added dc scenario with normal building opt
</commit_message>
<xml_diff>
--- a/Data/Charging_point_test_data.xlsx
+++ b/Data/Charging_point_test_data.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/araavind/Desktop/Python Files/LEC-Opt/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5773DA73-CFE8-9849-9891-BCF6454851A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4ECB79F-4900-A84B-B066-AD6D968202E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17180" xr2:uid="{D862B17B-82BE-45C1-B5E7-E58196152A87}"/>
+    <workbookView xWindow="-38400" yWindow="-1340" windowWidth="38400" windowHeight="19200" activeTab="4" xr2:uid="{D862B17B-82BE-45C1-B5E7-E58196152A87}"/>
   </bookViews>
   <sheets>
     <sheet name="CP1" sheetId="1" r:id="rId1"/>
     <sheet name="CP2" sheetId="2" r:id="rId2"/>
+    <sheet name="CP3" sheetId="3" r:id="rId3"/>
+    <sheet name="CP4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="7">
   <si>
     <t>Capacity</t>
   </si>
@@ -734,4 +737,522 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0086872-7C75-9142-AF94-C7F638E435C0}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>40</v>
+      </c>
+      <c r="B2">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1">
+        <v>44927.0625</v>
+      </c>
+      <c r="D2" s="1">
+        <v>44927.15625</v>
+      </c>
+      <c r="E2">
+        <v>0.87</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>90</v>
+      </c>
+      <c r="B3">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1">
+        <v>44927.166666666664</v>
+      </c>
+      <c r="D3" s="1">
+        <v>44927.71875</v>
+      </c>
+      <c r="E3">
+        <v>0.25</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>55</v>
+      </c>
+      <c r="B4">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1">
+        <v>44927.75</v>
+      </c>
+      <c r="D4" s="1">
+        <v>44927.927083333336</v>
+      </c>
+      <c r="E4">
+        <v>0.7</v>
+      </c>
+      <c r="F4">
+        <v>0.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5450018-935B-7B49-B596-CD804A9C2414}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="12.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>82</v>
+      </c>
+      <c r="B2">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1">
+        <v>44927.1875</v>
+      </c>
+      <c r="D2" s="1">
+        <v>44927.489583333336</v>
+      </c>
+      <c r="E2">
+        <v>0.74</v>
+      </c>
+      <c r="F2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>47</v>
+      </c>
+      <c r="B3">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1">
+        <v>44927.5</v>
+      </c>
+      <c r="D3" s="1">
+        <v>44927.84375</v>
+      </c>
+      <c r="E3">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>63</v>
+      </c>
+      <c r="B4">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1">
+        <v>44927.875</v>
+      </c>
+      <c r="D4" s="1">
+        <v>44927.927083333336</v>
+      </c>
+      <c r="E4">
+        <v>0.5</v>
+      </c>
+      <c r="F4">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B7FE47B-F1E9-2C4E-87F8-B8BDFF376642}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>50</v>
+      </c>
+      <c r="B2">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1">
+        <v>44927.041666666664</v>
+      </c>
+      <c r="D2" s="1">
+        <v>44927.208333333336</v>
+      </c>
+      <c r="E2">
+        <v>0.9</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>65</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>44927.291666666664</v>
+      </c>
+      <c r="D3" s="1">
+        <v>44927.625</v>
+      </c>
+      <c r="E3">
+        <v>0.8</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>70</v>
+      </c>
+      <c r="B4">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1">
+        <v>44927.75</v>
+      </c>
+      <c r="D4" s="1">
+        <v>44927.958333333336</v>
+      </c>
+      <c r="E4">
+        <v>0.7</v>
+      </c>
+      <c r="F4">
+        <v>0.8</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1">
+        <v>45047.604166666664</v>
+      </c>
+      <c r="D5" s="1">
+        <v>45078.708333333336</v>
+      </c>
+      <c r="E5">
+        <v>0.25</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>50</v>
+      </c>
+      <c r="B6">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1">
+        <v>44927.041666666664</v>
+      </c>
+      <c r="D6" s="1">
+        <v>44927.208333333336</v>
+      </c>
+      <c r="E6">
+        <v>0.7</v>
+      </c>
+      <c r="F6">
+        <v>0.8</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>65</v>
+      </c>
+      <c r="B7">
+        <v>7</v>
+      </c>
+      <c r="C7" s="1">
+        <v>44927.291666666664</v>
+      </c>
+      <c r="D7" s="1">
+        <v>44927.625</v>
+      </c>
+      <c r="E7">
+        <v>0.5</v>
+      </c>
+      <c r="F7">
+        <v>0.75</v>
+      </c>
+      <c r="G7">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>70</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1">
+        <v>44927.75</v>
+      </c>
+      <c r="D8" s="1">
+        <v>44927.958333333336</v>
+      </c>
+      <c r="E8">
+        <v>0.6</v>
+      </c>
+      <c r="F8">
+        <v>0.65</v>
+      </c>
+      <c r="G8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>40</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1">
+        <v>44927.0625</v>
+      </c>
+      <c r="D9" s="1">
+        <v>44927.15625</v>
+      </c>
+      <c r="E9">
+        <v>0.87</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>90</v>
+      </c>
+      <c r="B10">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1">
+        <v>44927.166666666664</v>
+      </c>
+      <c r="D10" s="1">
+        <v>44927.71875</v>
+      </c>
+      <c r="E10">
+        <v>0.25</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>55</v>
+      </c>
+      <c r="B11">
+        <v>7</v>
+      </c>
+      <c r="C11" s="1">
+        <v>44927.75</v>
+      </c>
+      <c r="D11" s="1">
+        <v>44927.927083333336</v>
+      </c>
+      <c r="E11">
+        <v>0.7</v>
+      </c>
+      <c r="F11">
+        <v>0.8</v>
+      </c>
+      <c r="G11">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>82</v>
+      </c>
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1">
+        <v>44927.1875</v>
+      </c>
+      <c r="D12" s="1">
+        <v>44927.489583333336</v>
+      </c>
+      <c r="E12">
+        <v>0.74</v>
+      </c>
+      <c r="F12">
+        <v>0.8</v>
+      </c>
+      <c r="G12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>47</v>
+      </c>
+      <c r="B13">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1">
+        <v>44927.5</v>
+      </c>
+      <c r="D13" s="1">
+        <v>44927.84375</v>
+      </c>
+      <c r="E13">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>63</v>
+      </c>
+      <c r="B14">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1">
+        <v>44927.875</v>
+      </c>
+      <c r="D14" s="1">
+        <v>44927.927083333336</v>
+      </c>
+      <c r="E14">
+        <v>0.5</v>
+      </c>
+      <c r="F14">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G14">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>